<commit_message>
edit words and phonemes
</commit_message>
<xml_diff>
--- a/yaml/Lexicon/Wordlists/verb.xlsx
+++ b/yaml/Lexicon/Wordlists/verb.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t xml:space="preserve">root</t>
   </si>
@@ -56,6 +56,30 @@
   </si>
   <si>
     <t xml:space="preserve">i_class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">want</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">be.able</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ganar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">win</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tomar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">take</t>
   </si>
 </sst>
 </file>
@@ -175,7 +199,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultColWidth="8.4296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -220,6 +244,50 @@
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>